<commit_message>
Use portable psql working directories
</commit_message>
<xml_diff>
--- a/task/关键标准答案.xlsx
+++ b/task/关键标准答案.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交付物答案清单" sheetId="1" r:id="R5c5508603b4d4af0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定字段答案" sheetId="2" r:id="Rc652265bd7e84836"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定集合答案" sheetId="3" r:id="Rb0def11079a14dee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定数值答案" sheetId="4" r:id="Rfed7b2783b3b4ca3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="允许变体答案" sheetId="5" r:id="R07f4959a7fbb4234"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交付物答案清单" sheetId="1" r:id="R16c157bb4df5437f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定字段答案" sheetId="2" r:id="Rdb2012ff143744c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定集合答案" sheetId="3" r:id="R9ae0c7a7aa4244e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定数值答案" sheetId="4" r:id="R2183cffc1bb244c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="允许变体答案" sheetId="5" r:id="Rbfb70bc9f6314bf6"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>